<commit_message>
docs: update summary and delete cache
</commit_message>
<xml_diff>
--- a/references/RedevSummary.xlsx
+++ b/references/RedevSummary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sapta\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sapta\Redev2026\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ED6904A-C615-4E12-BD61-261E9FC25354}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E42938A-75D2-4750-A8AA-5E021FA05DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -3172,6 +3172,27 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF991B1B"/>
       </font>
@@ -3198,27 +3219,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFDCFCE7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFD9EAD3"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5370,7 +5370,7 @@
         <v>604</v>
       </c>
       <c r="L2" s="4" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="M2" s="4"/>
     </row>
@@ -5407,7 +5407,7 @@
         <v>604</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>579</v>
+        <v>584</v>
       </c>
       <c r="M3" s="4"/>
     </row>
@@ -17867,13 +17867,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="L2:L337">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$L2="Done"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="4" priority="2">
       <formula>$L2="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="3" priority="3">
       <formula>$L2="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -19242,13 +19242,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E2:E49">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>E2="Done"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>E2="In Progress"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>E2="Blocked"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>